<commit_message>
Split user stories and sprint 1 user stories in Documents folder
</commit_message>
<xml_diff>
--- a/Documents/User_Stories/Sprint1_UserStories.xlsx
+++ b/Documents/User_Stories/Sprint1_UserStories.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoh\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danfox/dev/Old-Documents/Pace/Spring 2026/Computer Science Capstone Project/STARLABS/Documents/User_Stories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{83FC7195-7B22-4CCB-82B8-1407980F0286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACBA97DD-653E-7046-97AA-8F5E924F25F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8DDF8549-D73F-48F7-AEB6-DB20AE4C5F2F}"/>
+    <workbookView xWindow="-31300" yWindow="-5020" windowWidth="27500" windowHeight="15160" xr2:uid="{8DDF8549-D73F-48F7-AEB6-DB20AE4C5F2F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -411,25 +411,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
@@ -543,6 +524,55 @@
       </border>
     </dxf>
     <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -571,36 +601,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="medium">
-          <color rgb="FFCCCCCC"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top style="medium">
-          <color rgb="FFCCCCCC"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -615,12 +615,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{687F7A1C-14F1-4530-8A2B-FBF0A8BC9811}" name="Table1" displayName="Table1" ref="A1:E11" totalsRowShown="0" headerRowDxfId="6" dataDxfId="1" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{687F7A1C-14F1-4530-8A2B-FBF0A8BC9811}" name="Table1" displayName="Table1" ref="A1:E11" totalsRowShown="0" headerRowDxfId="9" dataDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="6" totalsRowBorderDxfId="5">
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{35B719C3-CB04-4C21-8D88-7FA3C4646BEB}" name="US_ID" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{FEB25D40-BA0D-4D4B-85CF-29D4CA7C72B5}" name="Feature" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{413A7D14-B8CD-48FF-A84C-C54746440881}" name="User Story" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{9711C4B5-5D93-40F9-B1B8-A9A48B911E4B}" name="Acceptance Criteria" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{35B719C3-CB04-4C21-8D88-7FA3C4646BEB}" name="US_ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{FEB25D40-BA0D-4D4B-85CF-29D4CA7C72B5}" name="Feature" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{413A7D14-B8CD-48FF-A84C-C54746440881}" name="User Story" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{9711C4B5-5D93-40F9-B1B8-A9A48B911E4B}" name="Acceptance Criteria" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{60B09A63-3608-4860-B064-FAC02AB4C087}" name="Story Points" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -628,9 +628,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -668,7 +668,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -774,7 +774,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -916,7 +916,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -925,16 +925,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{578F12B5-A4A3-4B64-BDDB-4651DECA0D18}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="93" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="93" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
     <col min="2" max="2" width="20.6640625" customWidth="1"/>
     <col min="3" max="3" width="51.33203125" customWidth="1"/>
-    <col min="4" max="4" width="61.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="21.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -951,7 +951,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="79.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="85" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -968,7 +968,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="85" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -985,7 +985,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="43" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="29" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="71" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="43" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="57" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
@@ -1070,7 +1070,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="66.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="71" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
@@ -1087,7 +1087,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="57" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="56" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>15</v>
       </c>

</xml_diff>